<commit_message>
feat(examples): enrich the showcase templates with more representative components
Add components a real corporate template carries, exercising extraction and the
now-broader generator:
- docx: a real external w:hyperlink in the body (a near-universal element the
  generator now also authors natively).
- pptx: speaker notes on the executive-summary slide (a standard deck artifact).
- xlsx: distributed-template sheet protection on Inputs with ONLY the input value
  cells (B4:B7) unlocked, plus a print header/footer with live fields (&[Tab],
  Page &P of &N).

All three rebuilt templates still extract with 0 schema problems and the
kitchen-sink + full suite stay green (264 passed, 4 skipped).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/templates/branddocs_template.xlsx
+++ b/examples/templates/branddocs_template.xlsx
@@ -168,7 +168,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
@@ -195,11 +195,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
@@ -1229,7 +1237,16 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1510,7 +1527,7 @@
           <t>Unit price (input)</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <f>Inputs!B5</f>
         <v/>
       </c>
@@ -1521,7 +1538,7 @@
           <t>Implied gross</t>
         </is>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <f>Inputs!B4*Inputs!B5</f>
         <v/>
       </c>
@@ -1532,7 +1549,7 @@
           <t>Net margin</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="18">
         <f>IF(B7=0,0,B4/B7)</f>
         <v/>
       </c>
@@ -1576,14 +1593,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Executive Dashboard</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Formula-backed snapshot generated from the model, inputs, and summary tabs</t>
         </is>
@@ -1612,19 +1629,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19">
+      <c r="A5" s="21">
         <f>Summary!B4</f>
         <v/>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="22">
         <f>Summary!B8</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="21">
         <f>Summary!B5</f>
         <v/>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="23">
         <f>Scenarios!B3</f>
         <v/>
       </c>
@@ -1797,10 +1814,10 @@
           <t>Base</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -1815,10 +1832,10 @@
           <t>Upside</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="24" t="n">
         <v>1.12</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="18" t="n">
         <v>0.025</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -1833,10 +1850,10 @@
           <t>Downside</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="24" t="n">
         <v>0.91</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="18" t="n">
         <v>-0.035</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -1935,7 +1952,7 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D2" s="23" t="n">
+      <c r="D2" s="25" t="n">
         <v>12500</v>
       </c>
     </row>
@@ -1955,7 +1972,7 @@
           <t>Gadget</t>
         </is>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="25" t="n">
         <v>9800</v>
       </c>
     </row>
@@ -1975,7 +1992,7 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="25" t="n">
         <v>14200</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(examples): one brand across the three example templates
The docx/pptx/xlsx builders had drifted apart on five supporting clrScheme
slots (three of them invented hexes), caught live by compare-profiles.
brand_theme_slots() in _brandlib is now the COMPLETE 12-slot map (the docx
reference values) and all three builders consume it verbatim; the pptx and
xlsx templates are regenerated byte-deterministically (the docx binary is
unchanged). compare-profiles on the shipped docx/pptx pair now reports
12/12 theme slots agreeing and matching theme fonts, pinned by a
strengthened CLI test that replaced the tautological verdict assertion.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/templates/branddocs_template.xlsx
+++ b/examples/templates/branddocs_template.xlsx
@@ -928,7 +928,7 @@
         <a:srgbClr val="16213F"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="EAF1FF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="2B7CD3"/>
@@ -946,19 +946,19 @@
         <a:srgbClr val="DCE7FF"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="5778B0"/>
+        <a:srgbClr val="E0742B"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="9CC0F0"/>
+        <a:srgbClr val="2B7CD3"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C7912B"/>
+        <a:srgbClr val="E0742B"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="2B7CD3"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="16213F"/>
+        <a:srgbClr val="E0742B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">

</xml_diff>